<commit_message>
Refresh slides, clean project files, and validate lecture figure scripts
</commit_message>
<xml_diff>
--- a/figures/lecture5/6345.0/634501.xlsx
+++ b/figures/lecture5/6345.0/634501.xlsx
@@ -17,89 +17,89 @@
     <sheet name="Enquiries" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="A2603039T">Data1!$B$1:$B$10,Data1!$B$11:$B$114</definedName>
-    <definedName name="A2603039T_Data">Data1!$B$11:$B$114</definedName>
-    <definedName name="A2603039T_Latest">Data1!$B$114</definedName>
-    <definedName name="A2603040A">Data1!$K$1:$K$10,Data1!$K$11:$K$114</definedName>
-    <definedName name="A2603040A_Data">Data1!$K$11:$K$114</definedName>
-    <definedName name="A2603040A_Latest">Data1!$K$114</definedName>
-    <definedName name="A2603041C">Data1!$T$1:$T$10,Data1!$T$11:$T$114</definedName>
-    <definedName name="A2603041C_Data">Data1!$T$11:$T$114</definedName>
-    <definedName name="A2603041C_Latest">Data1!$T$114</definedName>
-    <definedName name="A2603609J">Data1!$D$1:$D$10,Data1!$D$11:$D$114</definedName>
-    <definedName name="A2603609J_Data">Data1!$D$11:$D$114</definedName>
-    <definedName name="A2603609J_Latest">Data1!$D$114</definedName>
-    <definedName name="A2603610T">Data1!$M$1:$M$10,Data1!$M$11:$M$114</definedName>
-    <definedName name="A2603610T_Data">Data1!$M$11:$M$114</definedName>
-    <definedName name="A2603610T_Latest">Data1!$M$114</definedName>
-    <definedName name="A2603611V">Data1!$V$1:$V$10,Data1!$V$11:$V$114</definedName>
-    <definedName name="A2603611V_Data">Data1!$V$11:$V$114</definedName>
-    <definedName name="A2603611V_Latest">Data1!$V$114</definedName>
-    <definedName name="A2603989W">Data1!$C$1:$C$10,Data1!$C$11:$C$114</definedName>
-    <definedName name="A2603989W_Data">Data1!$C$11:$C$114</definedName>
-    <definedName name="A2603989W_Latest">Data1!$C$114</definedName>
-    <definedName name="A2603990F">Data1!$L$1:$L$10,Data1!$L$11:$L$114</definedName>
-    <definedName name="A2603990F_Data">Data1!$L$11:$L$114</definedName>
-    <definedName name="A2603990F_Latest">Data1!$L$114</definedName>
-    <definedName name="A2603991J">Data1!$U$1:$U$10,Data1!$U$11:$U$114</definedName>
-    <definedName name="A2603991J_Data">Data1!$U$11:$U$114</definedName>
-    <definedName name="A2603991J_Latest">Data1!$U$114</definedName>
-    <definedName name="A2713846W">Data1!$E$1:$E$10,Data1!$E$11:$E$114</definedName>
-    <definedName name="A2713846W_Data">Data1!$E$11:$E$114</definedName>
-    <definedName name="A2713846W_Latest">Data1!$E$114</definedName>
-    <definedName name="A2713848A">Data1!$H$1:$H$10,Data1!$H$11:$H$114</definedName>
-    <definedName name="A2713848A_Data">Data1!$H$11:$H$114</definedName>
-    <definedName name="A2713848A_Latest">Data1!$H$114</definedName>
-    <definedName name="A2713849C">Data1!$G$1:$G$10,Data1!$G$11:$G$114</definedName>
-    <definedName name="A2713849C_Data">Data1!$G$11:$G$114</definedName>
-    <definedName name="A2713849C_Latest">Data1!$G$114</definedName>
-    <definedName name="A2713851R">Data1!$J$1:$J$10,Data1!$J$11:$J$114</definedName>
-    <definedName name="A2713851R_Data">Data1!$J$11:$J$114</definedName>
-    <definedName name="A2713851R_Latest">Data1!$J$114</definedName>
-    <definedName name="A2713852T">Data1!$F$1:$F$10,Data1!$F$11:$F$114</definedName>
-    <definedName name="A2713852T_Data">Data1!$F$11:$F$114</definedName>
-    <definedName name="A2713852T_Latest">Data1!$F$114</definedName>
-    <definedName name="A2713854W">Data1!$I$1:$I$10,Data1!$I$11:$I$114</definedName>
-    <definedName name="A2713854W_Data">Data1!$I$11:$I$114</definedName>
-    <definedName name="A2713854W_Latest">Data1!$I$114</definedName>
-    <definedName name="A83895308K">Data1!$N$1:$N$10,Data1!$N$11:$N$114</definedName>
-    <definedName name="A83895308K_Data">Data1!$N$11:$N$114</definedName>
-    <definedName name="A83895308K_Latest">Data1!$N$114</definedName>
-    <definedName name="A83895309L">Data1!$W$1:$W$10,Data1!$W$11:$W$114</definedName>
-    <definedName name="A83895309L_Data">Data1!$W$11:$W$114</definedName>
-    <definedName name="A83895309L_Latest">Data1!$W$114</definedName>
-    <definedName name="A83895311X">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$114</definedName>
-    <definedName name="A83895311X_Data">Data1!$Q$11:$Q$114</definedName>
-    <definedName name="A83895311X_Latest">Data1!$Q$114</definedName>
-    <definedName name="A83895312A">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$114</definedName>
-    <definedName name="A83895312A_Data">Data1!$Z$11:$Z$114</definedName>
-    <definedName name="A83895312A_Latest">Data1!$Z$114</definedName>
-    <definedName name="A83895332K">Data1!$O$1:$O$10,Data1!$O$11:$O$114</definedName>
-    <definedName name="A83895332K_Data">Data1!$O$11:$O$114</definedName>
-    <definedName name="A83895332K_Latest">Data1!$O$114</definedName>
-    <definedName name="A83895333L">Data1!$X$1:$X$10,Data1!$X$11:$X$114</definedName>
-    <definedName name="A83895333L_Data">Data1!$X$11:$X$114</definedName>
-    <definedName name="A83895333L_Latest">Data1!$X$114</definedName>
-    <definedName name="A83895335T">Data1!$R$1:$R$10,Data1!$R$11:$R$114</definedName>
-    <definedName name="A83895335T_Data">Data1!$R$11:$R$114</definedName>
-    <definedName name="A83895335T_Latest">Data1!$R$114</definedName>
-    <definedName name="A83895336V">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$114</definedName>
-    <definedName name="A83895336V_Data">Data1!$AA$11:$AA$114</definedName>
-    <definedName name="A83895336V_Latest">Data1!$AA$114</definedName>
-    <definedName name="A83895395V">Data1!$P$1:$P$10,Data1!$P$11:$P$114</definedName>
-    <definedName name="A83895395V_Data">Data1!$P$11:$P$114</definedName>
-    <definedName name="A83895395V_Latest">Data1!$P$114</definedName>
-    <definedName name="A83895396W">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$114</definedName>
-    <definedName name="A83895396W_Data">Data1!$Y$11:$Y$114</definedName>
-    <definedName name="A83895396W_Latest">Data1!$Y$114</definedName>
-    <definedName name="A83895398A">Data1!$S$1:$S$10,Data1!$S$11:$S$114</definedName>
-    <definedName name="A83895398A_Data">Data1!$S$11:$S$114</definedName>
-    <definedName name="A83895398A_Latest">Data1!$S$114</definedName>
-    <definedName name="A83895399C">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$114</definedName>
-    <definedName name="A83895399C_Data">Data1!$AB$11:$AB$114</definedName>
-    <definedName name="A83895399C_Latest">Data1!$AB$114</definedName>
-    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$114</definedName>
-    <definedName name="Date_Range_Data">Data1!$A$11:$A$114</definedName>
+    <definedName name="A2603039T">Data1!$B$1:$B$10,Data1!$B$11:$B$124</definedName>
+    <definedName name="A2603039T_Data">Data1!$B$11:$B$124</definedName>
+    <definedName name="A2603039T_Latest">Data1!$B$124</definedName>
+    <definedName name="A2603040A">Data1!$K$1:$K$10,Data1!$K$11:$K$124</definedName>
+    <definedName name="A2603040A_Data">Data1!$K$11:$K$124</definedName>
+    <definedName name="A2603040A_Latest">Data1!$K$124</definedName>
+    <definedName name="A2603041C">Data1!$T$1:$T$10,Data1!$T$11:$T$124</definedName>
+    <definedName name="A2603041C_Data">Data1!$T$11:$T$124</definedName>
+    <definedName name="A2603041C_Latest">Data1!$T$124</definedName>
+    <definedName name="A2603609J">Data1!$D$1:$D$10,Data1!$D$11:$D$124</definedName>
+    <definedName name="A2603609J_Data">Data1!$D$11:$D$124</definedName>
+    <definedName name="A2603609J_Latest">Data1!$D$124</definedName>
+    <definedName name="A2603610T">Data1!$M$1:$M$10,Data1!$M$11:$M$124</definedName>
+    <definedName name="A2603610T_Data">Data1!$M$11:$M$124</definedName>
+    <definedName name="A2603610T_Latest">Data1!$M$124</definedName>
+    <definedName name="A2603611V">Data1!$V$1:$V$10,Data1!$V$11:$V$124</definedName>
+    <definedName name="A2603611V_Data">Data1!$V$11:$V$124</definedName>
+    <definedName name="A2603611V_Latest">Data1!$V$124</definedName>
+    <definedName name="A2603989W">Data1!$C$1:$C$10,Data1!$C$11:$C$124</definedName>
+    <definedName name="A2603989W_Data">Data1!$C$11:$C$124</definedName>
+    <definedName name="A2603989W_Latest">Data1!$C$124</definedName>
+    <definedName name="A2603990F">Data1!$L$1:$L$10,Data1!$L$11:$L$124</definedName>
+    <definedName name="A2603990F_Data">Data1!$L$11:$L$124</definedName>
+    <definedName name="A2603990F_Latest">Data1!$L$124</definedName>
+    <definedName name="A2603991J">Data1!$U$1:$U$10,Data1!$U$11:$U$124</definedName>
+    <definedName name="A2603991J_Data">Data1!$U$11:$U$124</definedName>
+    <definedName name="A2603991J_Latest">Data1!$U$124</definedName>
+    <definedName name="A2713846W">Data1!$E$1:$E$10,Data1!$E$11:$E$124</definedName>
+    <definedName name="A2713846W_Data">Data1!$E$11:$E$124</definedName>
+    <definedName name="A2713846W_Latest">Data1!$E$124</definedName>
+    <definedName name="A2713848A">Data1!$H$1:$H$10,Data1!$H$11:$H$124</definedName>
+    <definedName name="A2713848A_Data">Data1!$H$11:$H$124</definedName>
+    <definedName name="A2713848A_Latest">Data1!$H$124</definedName>
+    <definedName name="A2713849C">Data1!$G$1:$G$10,Data1!$G$11:$G$124</definedName>
+    <definedName name="A2713849C_Data">Data1!$G$11:$G$124</definedName>
+    <definedName name="A2713849C_Latest">Data1!$G$124</definedName>
+    <definedName name="A2713851R">Data1!$J$1:$J$10,Data1!$J$11:$J$124</definedName>
+    <definedName name="A2713851R_Data">Data1!$J$11:$J$124</definedName>
+    <definedName name="A2713851R_Latest">Data1!$J$124</definedName>
+    <definedName name="A2713852T">Data1!$F$1:$F$10,Data1!$F$11:$F$124</definedName>
+    <definedName name="A2713852T_Data">Data1!$F$11:$F$124</definedName>
+    <definedName name="A2713852T_Latest">Data1!$F$124</definedName>
+    <definedName name="A2713854W">Data1!$I$1:$I$10,Data1!$I$11:$I$124</definedName>
+    <definedName name="A2713854W_Data">Data1!$I$11:$I$124</definedName>
+    <definedName name="A2713854W_Latest">Data1!$I$124</definedName>
+    <definedName name="A83895308K">Data1!$N$1:$N$10,Data1!$N$11:$N$124</definedName>
+    <definedName name="A83895308K_Data">Data1!$N$11:$N$124</definedName>
+    <definedName name="A83895308K_Latest">Data1!$N$124</definedName>
+    <definedName name="A83895309L">Data1!$W$1:$W$10,Data1!$W$11:$W$124</definedName>
+    <definedName name="A83895309L_Data">Data1!$W$11:$W$124</definedName>
+    <definedName name="A83895309L_Latest">Data1!$W$124</definedName>
+    <definedName name="A83895311X">Data1!$Q$1:$Q$10,Data1!$Q$11:$Q$124</definedName>
+    <definedName name="A83895311X_Data">Data1!$Q$11:$Q$124</definedName>
+    <definedName name="A83895311X_Latest">Data1!$Q$124</definedName>
+    <definedName name="A83895312A">Data1!$Z$1:$Z$10,Data1!$Z$11:$Z$124</definedName>
+    <definedName name="A83895312A_Data">Data1!$Z$11:$Z$124</definedName>
+    <definedName name="A83895312A_Latest">Data1!$Z$124</definedName>
+    <definedName name="A83895332K">Data1!$O$1:$O$10,Data1!$O$11:$O$124</definedName>
+    <definedName name="A83895332K_Data">Data1!$O$11:$O$124</definedName>
+    <definedName name="A83895332K_Latest">Data1!$O$124</definedName>
+    <definedName name="A83895333L">Data1!$X$1:$X$10,Data1!$X$11:$X$124</definedName>
+    <definedName name="A83895333L_Data">Data1!$X$11:$X$124</definedName>
+    <definedName name="A83895333L_Latest">Data1!$X$124</definedName>
+    <definedName name="A83895335T">Data1!$R$1:$R$10,Data1!$R$11:$R$124</definedName>
+    <definedName name="A83895335T_Data">Data1!$R$11:$R$124</definedName>
+    <definedName name="A83895335T_Latest">Data1!$R$124</definedName>
+    <definedName name="A83895336V">Data1!$AA$1:$AA$10,Data1!$AA$11:$AA$124</definedName>
+    <definedName name="A83895336V_Data">Data1!$AA$11:$AA$124</definedName>
+    <definedName name="A83895336V_Latest">Data1!$AA$124</definedName>
+    <definedName name="A83895395V">Data1!$P$1:$P$10,Data1!$P$11:$P$124</definedName>
+    <definedName name="A83895395V_Data">Data1!$P$11:$P$124</definedName>
+    <definedName name="A83895395V_Latest">Data1!$P$124</definedName>
+    <definedName name="A83895396W">Data1!$Y$1:$Y$10,Data1!$Y$11:$Y$124</definedName>
+    <definedName name="A83895396W_Data">Data1!$Y$11:$Y$124</definedName>
+    <definedName name="A83895396W_Latest">Data1!$Y$124</definedName>
+    <definedName name="A83895398A">Data1!$S$1:$S$10,Data1!$S$11:$S$124</definedName>
+    <definedName name="A83895398A_Data">Data1!$S$11:$S$124</definedName>
+    <definedName name="A83895398A_Latest">Data1!$S$124</definedName>
+    <definedName name="A83895399C">Data1!$AB$1:$AB$10,Data1!$AB$11:$AB$124</definedName>
+    <definedName name="A83895399C_Data">Data1!$AB$11:$AB$124</definedName>
+    <definedName name="A83895399C_Latest">Data1!$AB$124</definedName>
+    <definedName name="Date_Range">Data1!$A$2:$A$10,Data1!$A$11:$A$124</definedName>
+    <definedName name="Date_Range_Data">Data1!$A$11:$A$124</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -1184,7 +1184,7 @@
     <t>Freq.</t>
   </si>
   <si>
-    <t>© Commonwealth of Australia  2023</t>
+    <t>© Commonwealth of Australia  2026</t>
   </si>
 </sst>
 </file>
@@ -1865,10 +1865,10 @@
         <v>35674</v>
       </c>
       <c r="G12" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H12" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I12" s="10" t="s">
         <v>24</v>
@@ -1897,10 +1897,10 @@
         <v>35674</v>
       </c>
       <c r="G13" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H13" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I13" s="10" t="s">
         <v>24</v>
@@ -1929,10 +1929,10 @@
         <v>35674</v>
       </c>
       <c r="G14" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H14" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I14" s="10" t="s">
         <v>24</v>
@@ -1961,10 +1961,10 @@
         <v>35674</v>
       </c>
       <c r="G15" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H15" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I15" s="10" t="s">
         <v>24</v>
@@ -1993,10 +1993,10 @@
         <v>35674</v>
       </c>
       <c r="G16" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H16" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I16" s="10" t="s">
         <v>24</v>
@@ -2025,10 +2025,10 @@
         <v>35674</v>
       </c>
       <c r="G17" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H17" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I17" s="10" t="s">
         <v>24</v>
@@ -2057,10 +2057,10 @@
         <v>35674</v>
       </c>
       <c r="G18" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H18" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I18" s="10" t="s">
         <v>24</v>
@@ -2089,10 +2089,10 @@
         <v>35674</v>
       </c>
       <c r="G19" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H19" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I19" s="10" t="s">
         <v>24</v>
@@ -2121,10 +2121,10 @@
         <v>35674</v>
       </c>
       <c r="G20" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H20" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I20" s="10" t="s">
         <v>24</v>
@@ -2153,10 +2153,10 @@
         <v>35674</v>
       </c>
       <c r="G21" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H21" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>39</v>
@@ -2185,10 +2185,10 @@
         <v>35674</v>
       </c>
       <c r="G22" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H22" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I22" s="10" t="s">
         <v>39</v>
@@ -2217,10 +2217,10 @@
         <v>35674</v>
       </c>
       <c r="G23" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H23" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I23" s="10" t="s">
         <v>39</v>
@@ -2249,10 +2249,10 @@
         <v>35674</v>
       </c>
       <c r="G24" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H24" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I24" s="10" t="s">
         <v>39</v>
@@ -2281,10 +2281,10 @@
         <v>35674</v>
       </c>
       <c r="G25" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H25" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I25" s="10" t="s">
         <v>39</v>
@@ -2313,10 +2313,10 @@
         <v>35674</v>
       </c>
       <c r="G26" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H26" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I26" s="10" t="s">
         <v>39</v>
@@ -2345,10 +2345,10 @@
         <v>35674</v>
       </c>
       <c r="G27" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H27" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I27" s="10" t="s">
         <v>39</v>
@@ -2377,10 +2377,10 @@
         <v>35674</v>
       </c>
       <c r="G28" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H28" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>39</v>
@@ -2409,10 +2409,10 @@
         <v>35674</v>
       </c>
       <c r="G29" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H29" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I29" s="10" t="s">
         <v>39</v>
@@ -2441,10 +2441,10 @@
         <v>35674</v>
       </c>
       <c r="G30" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H30" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I30" s="10" t="s">
         <v>39</v>
@@ -2473,10 +2473,10 @@
         <v>35674</v>
       </c>
       <c r="G31" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H31" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I31" s="10" t="s">
         <v>39</v>
@@ -2505,10 +2505,10 @@
         <v>35674</v>
       </c>
       <c r="G32" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H32" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>39</v>
@@ -2537,10 +2537,10 @@
         <v>35674</v>
       </c>
       <c r="G33" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H33" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I33" s="10" t="s">
         <v>39</v>
@@ -2569,10 +2569,10 @@
         <v>35674</v>
       </c>
       <c r="G34" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H34" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>39</v>
@@ -2601,10 +2601,10 @@
         <v>35674</v>
       </c>
       <c r="G35" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H35" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I35" s="10" t="s">
         <v>39</v>
@@ -2633,10 +2633,10 @@
         <v>35674</v>
       </c>
       <c r="G36" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H36" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I36" s="10" t="s">
         <v>39</v>
@@ -2665,10 +2665,10 @@
         <v>35674</v>
       </c>
       <c r="G37" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H37" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I37" s="10" t="s">
         <v>39</v>
@@ -2697,10 +2697,10 @@
         <v>35674</v>
       </c>
       <c r="G38" s="9">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H38" s="10">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I38" s="10" t="s">
         <v>39</v>
@@ -2762,7 +2762,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AB114"/>
+  <dimension ref="A1:AB124"/>
   <sheetFormatPr defaultColWidth="14.7109375" defaultRowHeight="11.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="16384" width="14.7109375" style="1"/>
@@ -3372,85 +3372,85 @@
         <v>21</v>
       </c>
       <c r="B8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="C8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="D8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="E8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="F8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="G8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="H8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="I8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="J8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="K8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="L8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="M8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="N8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="O8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="P8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="Q8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="R8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="S8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="T8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="U8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="V8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="W8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="X8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="Y8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="Z8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="AA8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
       <c r="AB8" s="6">
-        <v>45078</v>
+        <v>45992</v>
       </c>
     </row>
     <row r="9" spans="1:28" x14ac:dyDescent="0.2">
@@ -3458,85 +3458,85 @@
         <v>22</v>
       </c>
       <c r="B9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="C9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="D9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="E9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="F9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="G9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="H9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="I9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="J9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="K9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="L9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="M9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="N9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="O9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="P9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="Q9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="R9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="S9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="T9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="U9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="V9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="W9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="X9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="Y9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="Z9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="AA9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
       <c r="AB9" s="1">
-        <v>104</v>
+        <v>114</v>
       </c>
     </row>
     <row r="10" spans="1:28" x14ac:dyDescent="0.2">
@@ -5877,7 +5877,7 @@
         <v>82.3</v>
       </c>
       <c r="G38" s="8">
-        <v>83.1</v>
+        <v>83.2</v>
       </c>
       <c r="H38" s="8">
         <v>83.5</v>
@@ -5904,7 +5904,7 @@
         <v>0.9</v>
       </c>
       <c r="P38" s="8">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="Q38" s="8">
         <v>0.8</v>
@@ -5931,7 +5931,7 @@
         <v>4</v>
       </c>
       <c r="Y38" s="8">
-        <v>3.5</v>
+        <v>3.6</v>
       </c>
       <c r="Z38" s="8">
         <v>3.5</v>
@@ -5957,7 +5957,7 @@
         <v>84</v>
       </c>
       <c r="E39" s="8">
-        <v>84.2</v>
+        <v>84.1</v>
       </c>
       <c r="F39" s="8">
         <v>83.2</v>
@@ -5984,13 +5984,13 @@
         <v>1.3</v>
       </c>
       <c r="N39" s="8">
-        <v>0.8</v>
+        <v>0.7</v>
       </c>
       <c r="O39" s="8">
         <v>1.1000000000000001</v>
       </c>
       <c r="P39" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q39" s="8">
         <v>0.8</v>
@@ -6011,7 +6011,7 @@
         <v>3.6</v>
       </c>
       <c r="W39" s="8">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="X39" s="8">
         <v>3.9</v>
@@ -6070,7 +6070,7 @@
         <v>1</v>
       </c>
       <c r="N40" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O40" s="8">
         <v>1.2</v>
@@ -6129,7 +6129,7 @@
         <v>85.7</v>
       </c>
       <c r="E41" s="8">
-        <v>85.8</v>
+        <v>85.9</v>
       </c>
       <c r="F41" s="8">
         <v>85.3</v>
@@ -6156,7 +6156,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="N41" s="8">
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O41" s="8">
         <v>1.3</v>
@@ -6183,7 +6183,7 @@
         <v>3.9</v>
       </c>
       <c r="W41" s="8">
-        <v>3.6</v>
+        <v>3.7</v>
       </c>
       <c r="X41" s="8">
         <v>4.5</v>
@@ -6221,7 +6221,7 @@
         <v>86.2</v>
       </c>
       <c r="G42" s="8">
-        <v>86.5</v>
+        <v>86.6</v>
       </c>
       <c r="H42" s="8">
         <v>86.7</v>
@@ -6242,13 +6242,13 @@
         <v>0.7</v>
       </c>
       <c r="N42" s="8">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="O42" s="8">
         <v>1.1000000000000001</v>
       </c>
       <c r="P42" s="8">
-        <v>0.9</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Q42" s="8">
         <v>1</v>
@@ -6334,7 +6334,7 @@
         <v>1</v>
       </c>
       <c r="P43" s="8">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="Q43" s="8">
         <v>0.9</v>
@@ -6355,7 +6355,7 @@
         <v>4.2</v>
       </c>
       <c r="W43" s="8">
-        <v>3.9</v>
+        <v>4</v>
       </c>
       <c r="X43" s="8">
         <v>4.7</v>
@@ -6527,7 +6527,7 @@
         <v>4.0999999999999996</v>
       </c>
       <c r="W45" s="8">
-        <v>4.0999999999999996</v>
+        <v>4</v>
       </c>
       <c r="X45" s="8">
         <v>4.2</v>
@@ -6619,7 +6619,7 @@
         <v>4.3</v>
       </c>
       <c r="Y46" s="8">
-        <v>4.2</v>
+        <v>4</v>
       </c>
       <c r="Z46" s="8">
         <v>3.9</v>
@@ -6645,7 +6645,7 @@
         <v>90.9</v>
       </c>
       <c r="E47" s="8">
-        <v>91</v>
+        <v>90.9</v>
       </c>
       <c r="F47" s="8">
         <v>90.8</v>
@@ -6660,7 +6660,7 @@
         <v>90.9</v>
       </c>
       <c r="J47" s="8">
-        <v>90.9</v>
+        <v>91</v>
       </c>
       <c r="K47" s="8">
         <v>1</v>
@@ -6672,7 +6672,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="N47" s="8">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="O47" s="8">
         <v>1</v>
@@ -6687,7 +6687,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="S47" s="8">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="T47" s="8">
         <v>3.8</v>
@@ -6699,7 +6699,7 @@
         <v>3.9</v>
       </c>
       <c r="W47" s="8">
-        <v>4</v>
+        <v>3.9</v>
       </c>
       <c r="X47" s="8">
         <v>4.2</v>
@@ -6714,7 +6714,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="AB47" s="8">
-        <v>4</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="48" spans="1:28" x14ac:dyDescent="0.2">
@@ -6758,7 +6758,7 @@
         <v>1</v>
       </c>
       <c r="N48" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O48" s="8">
         <v>1.2</v>
@@ -6773,7 +6773,7 @@
         <v>1</v>
       </c>
       <c r="S48" s="8">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="T48" s="8">
         <v>3.7</v>
@@ -6918,7 +6918,7 @@
         <v>93.7</v>
       </c>
       <c r="J50" s="8">
-        <v>93.7</v>
+        <v>93.8</v>
       </c>
       <c r="K50" s="8">
         <v>0.9</v>
@@ -6945,7 +6945,7 @@
         <v>1</v>
       </c>
       <c r="S50" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="T50" s="8">
         <v>3.9</v>
@@ -6972,7 +6972,7 @@
         <v>4.2</v>
       </c>
       <c r="AB50" s="8">
-        <v>4</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="51" spans="1:28" x14ac:dyDescent="0.2">
@@ -6995,7 +6995,7 @@
         <v>94.7</v>
       </c>
       <c r="G51" s="8">
-        <v>94.7</v>
+        <v>94.8</v>
       </c>
       <c r="H51" s="8">
         <v>94.7</v>
@@ -7022,7 +7022,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="P51" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Q51" s="8">
         <v>1.1000000000000001</v>
@@ -7031,7 +7031,7 @@
         <v>1.1000000000000001</v>
       </c>
       <c r="S51" s="8">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="T51" s="8">
         <v>4.2</v>
@@ -7043,13 +7043,13 @@
         <v>4.3</v>
       </c>
       <c r="W51" s="8">
-        <v>4.0999999999999996</v>
+        <v>4.2</v>
       </c>
       <c r="X51" s="8">
         <v>4.3</v>
       </c>
       <c r="Y51" s="8">
-        <v>4.2</v>
+        <v>4.3</v>
       </c>
       <c r="Z51" s="8">
         <v>4.0999999999999996</v>
@@ -7058,7 +7058,7 @@
         <v>4.2</v>
       </c>
       <c r="AB51" s="8">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="52" spans="1:28" x14ac:dyDescent="0.2">
@@ -7108,7 +7108,7 @@
         <v>1</v>
       </c>
       <c r="P52" s="8">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q52" s="8">
         <v>1</v>
@@ -7167,7 +7167,7 @@
         <v>96.4</v>
       </c>
       <c r="G53" s="8">
-        <v>96.5</v>
+        <v>96.6</v>
       </c>
       <c r="H53" s="8">
         <v>96.7</v>
@@ -7194,7 +7194,7 @@
         <v>0.8</v>
       </c>
       <c r="P53" s="8">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="Q53" s="8">
         <v>1.2</v>
@@ -7221,7 +7221,7 @@
         <v>4</v>
       </c>
       <c r="Y53" s="8">
-        <v>4</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="Z53" s="8">
         <v>4.2</v>
@@ -7280,7 +7280,7 @@
         <v>0.9</v>
       </c>
       <c r="P54" s="8">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Q54" s="8">
         <v>1</v>
@@ -7316,7 +7316,7 @@
         <v>3.8</v>
       </c>
       <c r="AB54" s="8">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="55" spans="1:28" x14ac:dyDescent="0.2">
@@ -7339,7 +7339,7 @@
         <v>98.2</v>
       </c>
       <c r="G55" s="8">
-        <v>98.7</v>
+        <v>98.8</v>
       </c>
       <c r="H55" s="8">
         <v>98.8</v>
@@ -7366,7 +7366,7 @@
         <v>0.9</v>
       </c>
       <c r="P55" s="8">
-        <v>1</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="Q55" s="8">
         <v>1.1000000000000001</v>
@@ -7452,7 +7452,7 @@
         <v>1.4</v>
       </c>
       <c r="P56" s="8">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="Q56" s="8">
         <v>0.9</v>
@@ -7565,7 +7565,7 @@
         <v>4.4000000000000004</v>
       </c>
       <c r="Y57" s="8">
-        <v>4.2</v>
+        <v>4.0999999999999996</v>
       </c>
       <c r="Z57" s="8">
         <v>3.9</v>
@@ -7737,7 +7737,7 @@
         <v>4.5999999999999996</v>
       </c>
       <c r="Y59" s="8">
-        <v>3.1</v>
+        <v>3</v>
       </c>
       <c r="Z59" s="8">
         <v>2.8</v>
@@ -8371,7 +8371,7 @@
         <v>110.3</v>
       </c>
       <c r="G67" s="8">
-        <v>109.4</v>
+        <v>109.3</v>
       </c>
       <c r="H67" s="8">
         <v>109.1</v>
@@ -8398,7 +8398,7 @@
         <v>0.6</v>
       </c>
       <c r="P67" s="8">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Q67" s="8">
         <v>0.9</v>
@@ -8425,7 +8425,7 @@
         <v>3.3</v>
       </c>
       <c r="Y67" s="8">
-        <v>3.7</v>
+        <v>3.6</v>
       </c>
       <c r="Z67" s="8">
         <v>3.8</v>
@@ -8484,7 +8484,7 @@
         <v>0.8</v>
       </c>
       <c r="P68" s="8">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="Q68" s="8">
         <v>1</v>
@@ -8769,7 +8769,7 @@
         <v>3.4</v>
       </c>
       <c r="Y71" s="8">
-        <v>3.7</v>
+        <v>3.8</v>
       </c>
       <c r="Z71" s="8">
         <v>3.7</v>
@@ -10865,7 +10865,7 @@
         <v>133.6</v>
       </c>
       <c r="G96" s="8">
-        <v>130.6</v>
+        <v>130.5</v>
       </c>
       <c r="H96" s="8">
         <v>129.69999999999999</v>
@@ -10892,7 +10892,7 @@
         <v>0.7</v>
       </c>
       <c r="P96" s="8">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="Q96" s="8">
         <v>0.6</v>
@@ -10919,7 +10919,7 @@
         <v>2.5</v>
       </c>
       <c r="Y96" s="8">
-        <v>2.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Z96" s="8">
         <v>2.2999999999999998</v>
@@ -11034,7 +11034,7 @@
         <v>131.1</v>
       </c>
       <c r="F98" s="8">
-        <v>135.1</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="G98" s="8">
         <v>132</v>
@@ -11061,7 +11061,7 @@
         <v>0.5</v>
       </c>
       <c r="O98" s="8">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="P98" s="8">
         <v>0.6</v>
@@ -11088,7 +11088,7 @@
         <v>2.2999999999999998</v>
       </c>
       <c r="X98" s="8">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="Y98" s="8">
         <v>2.2999999999999998</v>
@@ -11147,7 +11147,7 @@
         <v>0.5</v>
       </c>
       <c r="O99" s="8">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="P99" s="8">
         <v>0.5</v>
@@ -11263,7 +11263,7 @@
         <v>2.2000000000000002</v>
       </c>
       <c r="Y100" s="8">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="Z100" s="8">
         <v>2.2000000000000002</v>
@@ -11292,7 +11292,7 @@
         <v>133.19999999999999</v>
       </c>
       <c r="F101" s="8">
-        <v>137.30000000000001</v>
+        <v>137.19999999999999</v>
       </c>
       <c r="G101" s="8">
         <v>134.1</v>
@@ -11319,7 +11319,7 @@
         <v>0.5</v>
       </c>
       <c r="O101" s="8">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="P101" s="8">
         <v>0.5</v>
@@ -11346,7 +11346,7 @@
         <v>2.1</v>
       </c>
       <c r="X101" s="8">
-        <v>2.4</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="Y101" s="8">
         <v>2.2000000000000002</v>
@@ -11375,7 +11375,7 @@
         <v>134.1</v>
       </c>
       <c r="E102" s="8">
-        <v>133.30000000000001</v>
+        <v>133.4</v>
       </c>
       <c r="F102" s="8">
         <v>138</v>
@@ -11402,10 +11402,10 @@
         <v>0</v>
       </c>
       <c r="N102" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="O102" s="8">
-        <v>0.5</v>
+        <v>0.6</v>
       </c>
       <c r="P102" s="8">
         <v>0.2</v>
@@ -11429,7 +11429,7 @@
         <v>1.7</v>
       </c>
       <c r="W102" s="8">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="X102" s="8">
         <v>2.1</v>
@@ -11467,7 +11467,7 @@
         <v>138.4</v>
       </c>
       <c r="G103" s="8">
-        <v>134.6</v>
+        <v>134.5</v>
       </c>
       <c r="H103" s="8">
         <v>133.9</v>
@@ -11488,7 +11488,7 @@
         <v>0.4</v>
       </c>
       <c r="N103" s="8">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="O103" s="8">
         <v>0.3</v>
@@ -11547,13 +11547,13 @@
         <v>135.4</v>
       </c>
       <c r="E104" s="8">
-        <v>134.30000000000001</v>
+        <v>134.19999999999999</v>
       </c>
       <c r="F104" s="8">
         <v>138.69999999999999</v>
       </c>
       <c r="G104" s="8">
-        <v>135.30000000000001</v>
+        <v>135.19999999999999</v>
       </c>
       <c r="H104" s="8">
         <v>134.5</v>
@@ -11574,7 +11574,7 @@
         <v>0.5</v>
       </c>
       <c r="N104" s="8">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="O104" s="8">
         <v>0.2</v>
@@ -11601,13 +11601,13 @@
         <v>1.4</v>
       </c>
       <c r="W104" s="8">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="X104" s="8">
         <v>1.6</v>
       </c>
       <c r="Y104" s="8">
-        <v>1.4</v>
+        <v>1.3</v>
       </c>
       <c r="Z104" s="8">
         <v>1.5</v>
@@ -11639,7 +11639,7 @@
         <v>139.30000000000001</v>
       </c>
       <c r="G105" s="8">
-        <v>136</v>
+        <v>136.1</v>
       </c>
       <c r="H105" s="8">
         <v>135.1</v>
@@ -11666,7 +11666,7 @@
         <v>0.4</v>
       </c>
       <c r="P105" s="8">
-        <v>0.5</v>
+        <v>0.7</v>
       </c>
       <c r="Q105" s="8">
         <v>0.4</v>
@@ -11693,7 +11693,7 @@
         <v>1.5</v>
       </c>
       <c r="Y105" s="8">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
       <c r="Z105" s="8">
         <v>1.4</v>
@@ -11719,7 +11719,7 @@
         <v>136.5</v>
       </c>
       <c r="E106" s="8">
-        <v>135.80000000000001</v>
+        <v>135.9</v>
       </c>
       <c r="F106" s="8">
         <v>139.80000000000001</v>
@@ -11746,13 +11746,13 @@
         <v>0.3</v>
       </c>
       <c r="N106" s="8">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="O106" s="8">
         <v>0.4</v>
       </c>
       <c r="P106" s="8">
-        <v>0.6</v>
+        <v>0.5</v>
       </c>
       <c r="Q106" s="8">
         <v>0.5</v>
@@ -11832,7 +11832,7 @@
         <v>0.9</v>
       </c>
       <c r="N107" s="8">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="O107" s="8">
         <v>0.6</v>
@@ -11891,10 +11891,10 @@
         <v>138.5</v>
       </c>
       <c r="E108" s="8">
-        <v>137.5</v>
+        <v>137.4</v>
       </c>
       <c r="F108" s="8">
-        <v>141.69999999999999</v>
+        <v>141.6</v>
       </c>
       <c r="G108" s="8">
         <v>138.4</v>
@@ -11903,7 +11903,7 @@
         <v>137.4</v>
       </c>
       <c r="I108" s="8">
-        <v>141.6</v>
+        <v>141.5</v>
       </c>
       <c r="J108" s="8">
         <v>138.30000000000001</v>
@@ -11921,7 +11921,7 @@
         <v>0.7</v>
       </c>
       <c r="O108" s="8">
-        <v>0.7</v>
+        <v>0.6</v>
       </c>
       <c r="P108" s="8">
         <v>0.7</v>
@@ -11948,16 +11948,16 @@
         <v>2.4</v>
       </c>
       <c r="X108" s="8">
-        <v>2.2000000000000002</v>
+        <v>2.1</v>
       </c>
       <c r="Y108" s="8">
-        <v>2.2999999999999998</v>
+        <v>2.4</v>
       </c>
       <c r="Z108" s="8">
         <v>2.2000000000000002</v>
       </c>
       <c r="AA108" s="8">
-        <v>2</v>
+        <v>1.9</v>
       </c>
       <c r="AB108" s="8">
         <v>2.2000000000000002</v>
@@ -11980,10 +11980,10 @@
         <v>138.4</v>
       </c>
       <c r="F109" s="8">
-        <v>142.4</v>
+        <v>142.30000000000001</v>
       </c>
       <c r="G109" s="8">
-        <v>139.19999999999999</v>
+        <v>139.30000000000001</v>
       </c>
       <c r="H109" s="8">
         <v>138.4</v>
@@ -12010,7 +12010,7 @@
         <v>0.5</v>
       </c>
       <c r="P109" s="8">
-        <v>0.6</v>
+        <v>0.7</v>
       </c>
       <c r="Q109" s="8">
         <v>0.7</v>
@@ -12063,7 +12063,7 @@
         <v>140.1</v>
       </c>
       <c r="E110" s="8">
-        <v>139.5</v>
+        <v>139.6</v>
       </c>
       <c r="F110" s="8">
         <v>143.19999999999999</v>
@@ -12090,13 +12090,13 @@
         <v>0.6</v>
       </c>
       <c r="N110" s="8">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="O110" s="8">
         <v>0.6</v>
       </c>
       <c r="P110" s="8">
-        <v>0.9</v>
+        <v>0.8</v>
       </c>
       <c r="Q110" s="8">
         <v>0.9</v>
@@ -12149,22 +12149,22 @@
         <v>142.1</v>
       </c>
       <c r="E111" s="8">
-        <v>141.19999999999999</v>
+        <v>141.1</v>
       </c>
       <c r="F111" s="8">
         <v>144.1</v>
       </c>
       <c r="G111" s="8">
-        <v>141.9</v>
+        <v>141.80000000000001</v>
       </c>
       <c r="H111" s="8">
-        <v>141.1</v>
+        <v>141</v>
       </c>
       <c r="I111" s="8">
         <v>144.1</v>
       </c>
       <c r="J111" s="8">
-        <v>141.80000000000001</v>
+        <v>141.69999999999999</v>
       </c>
       <c r="K111" s="8">
         <v>1.7</v>
@@ -12176,16 +12176,16 @@
         <v>1.4</v>
       </c>
       <c r="N111" s="8">
-        <v>1.2</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="O111" s="8">
         <v>0.6</v>
       </c>
       <c r="P111" s="8">
-        <v>1.1000000000000001</v>
+        <v>1</v>
       </c>
       <c r="Q111" s="8">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="R111" s="8">
         <v>0.6</v>
@@ -12209,10 +12209,10 @@
         <v>2.4</v>
       </c>
       <c r="Y111" s="8">
+        <v>3.1</v>
+      </c>
+      <c r="Z111" s="8">
         <v>3.2</v>
-      </c>
-      <c r="Z111" s="8">
-        <v>3.3</v>
       </c>
       <c r="AA111" s="8">
         <v>2.4</v>
@@ -12235,22 +12235,22 @@
         <v>143.19999999999999</v>
       </c>
       <c r="E112" s="8">
-        <v>142.5</v>
+        <v>142.4</v>
       </c>
       <c r="F112" s="8">
         <v>145.19999999999999</v>
       </c>
       <c r="G112" s="8">
-        <v>143.1</v>
+        <v>143</v>
       </c>
       <c r="H112" s="8">
         <v>142.4</v>
       </c>
       <c r="I112" s="8">
-        <v>145.30000000000001</v>
+        <v>145.19999999999999</v>
       </c>
       <c r="J112" s="8">
-        <v>143.1</v>
+        <v>143</v>
       </c>
       <c r="K112" s="8">
         <v>0.8</v>
@@ -12271,7 +12271,7 @@
         <v>0.8</v>
       </c>
       <c r="Q112" s="8">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="R112" s="8">
         <v>0.8</v>
@@ -12295,7 +12295,7 @@
         <v>2.5</v>
       </c>
       <c r="Y112" s="8">
-        <v>3.4</v>
+        <v>3.3</v>
       </c>
       <c r="Z112" s="8">
         <v>3.6</v>
@@ -12304,7 +12304,7 @@
         <v>2.6</v>
       </c>
       <c r="AB112" s="8">
-        <v>3.5</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="113" spans="1:28" x14ac:dyDescent="0.2">
@@ -12324,10 +12324,10 @@
         <v>143.69999999999999</v>
       </c>
       <c r="F113" s="8">
-        <v>146.6</v>
+        <v>146.5</v>
       </c>
       <c r="G113" s="8">
-        <v>144.30000000000001</v>
+        <v>144.4</v>
       </c>
       <c r="H113" s="8">
         <v>143.69999999999999</v>
@@ -12348,14 +12348,14 @@
         <v>0.8</v>
       </c>
       <c r="N113" s="8">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="O113" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="P113" s="8">
         <v>1</v>
       </c>
-      <c r="P113" s="8">
-        <v>0.8</v>
-      </c>
       <c r="Q113" s="8">
         <v>0.9</v>
       </c>
@@ -12363,7 +12363,7 @@
         <v>0.8</v>
       </c>
       <c r="S113" s="8">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="T113" s="8">
         <v>3.8</v>
@@ -12378,7 +12378,7 @@
         <v>3.8</v>
       </c>
       <c r="X113" s="8">
-        <v>2.9</v>
+        <v>3</v>
       </c>
       <c r="Y113" s="8">
         <v>3.7</v>
@@ -12407,22 +12407,22 @@
         <v>145.19999999999999</v>
       </c>
       <c r="E114" s="8">
-        <v>144.80000000000001</v>
+        <v>145</v>
       </c>
       <c r="F114" s="8">
         <v>147.6</v>
       </c>
       <c r="G114" s="8">
-        <v>145.5</v>
+        <v>145.6</v>
       </c>
       <c r="H114" s="8">
-        <v>144.80000000000001</v>
+        <v>145.19999999999999</v>
       </c>
       <c r="I114" s="8">
-        <v>147.6</v>
+        <v>147.80000000000001</v>
       </c>
       <c r="J114" s="8">
-        <v>145.5</v>
+        <v>145.80000000000001</v>
       </c>
       <c r="K114" s="8">
         <v>0.6</v>
@@ -12434,22 +12434,22 @@
         <v>0.6</v>
       </c>
       <c r="N114" s="8">
-        <v>0.8</v>
+        <v>0.9</v>
       </c>
       <c r="O114" s="8">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="P114" s="8">
         <v>0.8</v>
       </c>
       <c r="Q114" s="8">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="R114" s="8">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="S114" s="8">
-        <v>0.8</v>
+        <v>1</v>
       </c>
       <c r="T114" s="8">
         <v>3.8</v>
@@ -12461,22 +12461,882 @@
         <v>3.6</v>
       </c>
       <c r="W114" s="8">
-        <v>3.8</v>
+        <v>3.9</v>
       </c>
       <c r="X114" s="8">
         <v>3.1</v>
       </c>
       <c r="Y114" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="Z114" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="AA114" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="AB114" s="8">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="115" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A115" s="9">
+        <v>45170</v>
+      </c>
+      <c r="B115" s="8">
+        <v>147.5</v>
+      </c>
+      <c r="C115" s="8">
+        <v>149.1</v>
+      </c>
+      <c r="D115" s="8">
+        <v>147.9</v>
+      </c>
+      <c r="E115" s="8">
+        <v>147.1</v>
+      </c>
+      <c r="F115" s="8">
+        <v>149.19999999999999</v>
+      </c>
+      <c r="G115" s="8">
+        <v>147.5</v>
+      </c>
+      <c r="H115" s="8">
+        <v>146.9</v>
+      </c>
+      <c r="I115" s="8">
+        <v>149.4</v>
+      </c>
+      <c r="J115" s="8">
+        <v>147.4</v>
+      </c>
+      <c r="K115" s="8">
+        <v>2.1</v>
+      </c>
+      <c r="L115" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M115" s="8">
+        <v>1.9</v>
+      </c>
+      <c r="N115" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="O115" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="P115" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="Q115" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="R115" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="S115" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="T115" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="U115" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="V115" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="W115" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="X115" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="Y115" s="8">
+        <v>4</v>
+      </c>
+      <c r="Z115" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="AA115" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="AB115" s="8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="116" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A116" s="9">
+        <v>45261</v>
+      </c>
+      <c r="B116" s="8">
+        <v>148.6</v>
+      </c>
+      <c r="C116" s="8">
+        <v>151.4</v>
+      </c>
+      <c r="D116" s="8">
+        <v>149.30000000000001</v>
+      </c>
+      <c r="E116" s="8">
+        <v>148.4</v>
+      </c>
+      <c r="F116" s="8">
+        <v>151.4</v>
+      </c>
+      <c r="G116" s="8">
+        <v>149.1</v>
+      </c>
+      <c r="H116" s="8">
+        <v>148.4</v>
+      </c>
+      <c r="I116" s="8">
+        <v>150.9</v>
+      </c>
+      <c r="J116" s="8">
+        <v>149</v>
+      </c>
+      <c r="K116" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="L116" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="M116" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="N116" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="O116" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="P116" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="Q116" s="8">
+        <v>1</v>
+      </c>
+      <c r="R116" s="8">
+        <v>1</v>
+      </c>
+      <c r="S116" s="8">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="T116" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="U116" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="V116" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="W116" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="X116" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="Y116" s="8">
+        <v>4.3</v>
+      </c>
+      <c r="Z116" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="AA116" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="AB116" s="8">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="117" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A117" s="9">
+        <v>45352</v>
+      </c>
+      <c r="B117" s="8">
+        <v>149.5</v>
+      </c>
+      <c r="C117" s="8">
+        <v>152.19999999999999</v>
+      </c>
+      <c r="D117" s="8">
+        <v>150.19999999999999</v>
+      </c>
+      <c r="E117" s="8">
+        <v>149.69999999999999</v>
+      </c>
+      <c r="F117" s="8">
+        <v>152</v>
+      </c>
+      <c r="G117" s="8">
+        <v>150.19999999999999</v>
+      </c>
+      <c r="H117" s="8">
+        <v>149.69999999999999</v>
+      </c>
+      <c r="I117" s="8">
+        <v>152.30000000000001</v>
+      </c>
+      <c r="J117" s="8">
+        <v>150.30000000000001</v>
+      </c>
+      <c r="K117" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="L117" s="8">
+        <v>0.5</v>
+      </c>
+      <c r="M117" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="N117" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="O117" s="8">
+        <v>0.4</v>
+      </c>
+      <c r="P117" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="Q117" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="R117" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="S117" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="T117" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="U117" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="V117" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="W117" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="X117" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="Y117" s="8">
+        <v>4</v>
+      </c>
+      <c r="Z117" s="8">
+        <v>4.2</v>
+      </c>
+      <c r="AA117" s="8">
+        <v>4</v>
+      </c>
+      <c r="AB117" s="8">
+        <v>4.2</v>
+      </c>
+    </row>
+    <row r="118" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A118" s="9">
+        <v>45444</v>
+      </c>
+      <c r="B118" s="8">
+        <v>150.4</v>
+      </c>
+      <c r="C118" s="8">
+        <v>153.30000000000001</v>
+      </c>
+      <c r="D118" s="8">
+        <v>151.1</v>
+      </c>
+      <c r="E118" s="8">
+        <v>150.9</v>
+      </c>
+      <c r="F118" s="8">
+        <v>153.5</v>
+      </c>
+      <c r="G118" s="8">
+        <v>151.5</v>
+      </c>
+      <c r="H118" s="8">
+        <v>150.9</v>
+      </c>
+      <c r="I118" s="8">
+        <v>153.4</v>
+      </c>
+      <c r="J118" s="8">
+        <v>151.5</v>
+      </c>
+      <c r="K118" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="L118" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="M118" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="N118" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="O118" s="8">
+        <v>1</v>
+      </c>
+      <c r="P118" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="Q118" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R118" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="S118" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="T118" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="U118" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="V118" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="W118" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="X118" s="8">
+        <v>4</v>
+      </c>
+      <c r="Y118" s="8">
+        <v>4.0999999999999996</v>
+      </c>
+      <c r="Z118" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="AA118" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="AB118" s="8">
+        <v>3.9</v>
+      </c>
+    </row>
+    <row r="119" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A119" s="9">
+        <v>45536</v>
+      </c>
+      <c r="B119" s="8">
+        <v>152.6</v>
+      </c>
+      <c r="C119" s="8">
+        <v>154.6</v>
+      </c>
+      <c r="D119" s="8">
+        <v>153.1</v>
+      </c>
+      <c r="E119" s="8">
+        <v>152.19999999999999</v>
+      </c>
+      <c r="F119" s="8">
+        <v>154.6</v>
+      </c>
+      <c r="G119" s="8">
+        <v>152.80000000000001</v>
+      </c>
+      <c r="H119" s="8">
+        <v>152.19999999999999</v>
+      </c>
+      <c r="I119" s="8">
+        <v>154.6</v>
+      </c>
+      <c r="J119" s="8">
+        <v>152.69999999999999</v>
+      </c>
+      <c r="K119" s="8">
+        <v>1.5</v>
+      </c>
+      <c r="L119" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="M119" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="N119" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="O119" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="P119" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="Q119" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="R119" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="S119" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="T119" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="U119" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="V119" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="W119" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="X119" s="8">
         <v>3.6</v>
       </c>
-      <c r="Z114" s="8">
+      <c r="Y119" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="Z119" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="AA119" s="8">
+        <v>3.5</v>
+      </c>
+      <c r="AB119" s="8">
+        <v>3.6</v>
+      </c>
+    </row>
+    <row r="120" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A120" s="9">
+        <v>45627</v>
+      </c>
+      <c r="B120" s="8">
+        <v>153.6</v>
+      </c>
+      <c r="C120" s="8">
+        <v>155.80000000000001</v>
+      </c>
+      <c r="D120" s="8">
+        <v>154.1</v>
+      </c>
+      <c r="E120" s="8">
+        <v>153.30000000000001</v>
+      </c>
+      <c r="F120" s="8">
+        <v>155.69999999999999</v>
+      </c>
+      <c r="G120" s="8">
+        <v>153.9</v>
+      </c>
+      <c r="H120" s="8">
+        <v>153.4</v>
+      </c>
+      <c r="I120" s="8">
+        <v>155.9</v>
+      </c>
+      <c r="J120" s="8">
+        <v>154</v>
+      </c>
+      <c r="K120" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="L120" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="M120" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="N120" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="O120" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="P120" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="Q120" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R120" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="S120" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="T120" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="U120" s="8">
+        <v>2.9</v>
+      </c>
+      <c r="V120" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="W120" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="X120" s="8">
+        <v>2.8</v>
+      </c>
+      <c r="Y120" s="8">
+        <v>3.2</v>
+      </c>
+      <c r="Z120" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="AA120" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AB120" s="8">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="121" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A121" s="9">
+        <v>45717</v>
+      </c>
+      <c r="B121" s="8">
+        <v>154.5</v>
+      </c>
+      <c r="C121" s="8">
+        <v>157.69999999999999</v>
+      </c>
+      <c r="D121" s="8">
+        <v>155.30000000000001</v>
+      </c>
+      <c r="E121" s="8">
+        <v>154.69999999999999</v>
+      </c>
+      <c r="F121" s="8">
+        <v>157.5</v>
+      </c>
+      <c r="G121" s="8">
+        <v>155.30000000000001</v>
+      </c>
+      <c r="H121" s="8">
+        <v>154.69999999999999</v>
+      </c>
+      <c r="I121" s="8">
+        <v>157.4</v>
+      </c>
+      <c r="J121" s="8">
+        <v>155.30000000000001</v>
+      </c>
+      <c r="K121" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="L121" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="M121" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="N121" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="O121" s="8">
+        <v>1.2</v>
+      </c>
+      <c r="P121" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="Q121" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R121" s="8">
+        <v>1</v>
+      </c>
+      <c r="S121" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="T121" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="U121" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="V121" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="W121" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="X121" s="8">
+        <v>3.6</v>
+      </c>
+      <c r="Y121" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="Z121" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AA121" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AB121" s="8">
+        <v>3.3</v>
+      </c>
+    </row>
+    <row r="122" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A122" s="9">
+        <v>45809</v>
+      </c>
+      <c r="B122" s="8">
+        <v>155.4</v>
+      </c>
+      <c r="C122" s="8">
+        <v>158.9</v>
+      </c>
+      <c r="D122" s="8">
+        <v>156.19999999999999</v>
+      </c>
+      <c r="E122" s="8">
+        <v>156</v>
+      </c>
+      <c r="F122" s="8">
+        <v>159.1</v>
+      </c>
+      <c r="G122" s="8">
+        <v>156.69999999999999</v>
+      </c>
+      <c r="H122" s="8">
+        <v>155.9</v>
+      </c>
+      <c r="I122" s="8">
+        <v>159</v>
+      </c>
+      <c r="J122" s="8">
+        <v>156.6</v>
+      </c>
+      <c r="K122" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="L122" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="M122" s="8">
+        <v>0.6</v>
+      </c>
+      <c r="N122" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="O122" s="8">
+        <v>1</v>
+      </c>
+      <c r="P122" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="Q122" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R122" s="8">
+        <v>1</v>
+      </c>
+      <c r="S122" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="T122" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="U122" s="8">
         <v>3.7</v>
       </c>
-      <c r="AA114" s="8">
-        <v>3.1</v>
-      </c>
-      <c r="AB114" s="8">
+      <c r="V122" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="W122" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="X122" s="8">
         <v>3.6</v>
+      </c>
+      <c r="Y122" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="Z122" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AA122" s="8">
+        <v>3.7</v>
+      </c>
+      <c r="AB122" s="8">
+        <v>3.4</v>
+      </c>
+    </row>
+    <row r="123" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A123" s="9">
+        <v>45901</v>
+      </c>
+      <c r="B123" s="8">
+        <v>157.6</v>
+      </c>
+      <c r="C123" s="8">
+        <v>160.5</v>
+      </c>
+      <c r="D123" s="8">
+        <v>158.30000000000001</v>
+      </c>
+      <c r="E123" s="8">
+        <v>157.19999999999999</v>
+      </c>
+      <c r="F123" s="8">
+        <v>160.6</v>
+      </c>
+      <c r="G123" s="8">
+        <v>157.9</v>
+      </c>
+      <c r="H123" s="8">
+        <v>157.19999999999999</v>
+      </c>
+      <c r="I123" s="8">
+        <v>160.5</v>
+      </c>
+      <c r="J123" s="8">
+        <v>158</v>
+      </c>
+      <c r="K123" s="8">
+        <v>1.4</v>
+      </c>
+      <c r="L123" s="8">
+        <v>1</v>
+      </c>
+      <c r="M123" s="8">
+        <v>1.3</v>
+      </c>
+      <c r="N123" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="O123" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="P123" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="Q123" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R123" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="S123" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="T123" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="U123" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="V123" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="W123" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="X123" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="Y123" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="Z123" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AA123" s="8">
+        <v>3.8</v>
+      </c>
+      <c r="AB123" s="8">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="124" spans="1:28" x14ac:dyDescent="0.2">
+      <c r="A124" s="9">
+        <v>45992</v>
+      </c>
+      <c r="B124" s="8">
+        <v>158.69999999999999</v>
+      </c>
+      <c r="C124" s="8">
+        <v>161.9</v>
+      </c>
+      <c r="D124" s="8">
+        <v>159.4</v>
+      </c>
+      <c r="E124" s="8">
+        <v>158.5</v>
+      </c>
+      <c r="F124" s="8">
+        <v>161.9</v>
+      </c>
+      <c r="G124" s="8">
+        <v>159.19999999999999</v>
+      </c>
+      <c r="H124" s="8">
+        <v>158.4</v>
+      </c>
+      <c r="I124" s="8">
+        <v>162</v>
+      </c>
+      <c r="J124" s="8">
+        <v>159.19999999999999</v>
+      </c>
+      <c r="K124" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="L124" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="M124" s="8">
+        <v>0.7</v>
+      </c>
+      <c r="N124" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="O124" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="P124" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="Q124" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="R124" s="8">
+        <v>0.9</v>
+      </c>
+      <c r="S124" s="8">
+        <v>0.8</v>
+      </c>
+      <c r="T124" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="U124" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="V124" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="W124" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="X124" s="8">
+        <v>4</v>
+      </c>
+      <c r="Y124" s="8">
+        <v>3.4</v>
+      </c>
+      <c r="Z124" s="8">
+        <v>3.3</v>
+      </c>
+      <c r="AA124" s="8">
+        <v>3.9</v>
+      </c>
+      <c r="AB124" s="8">
+        <v>3.4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>